<commit_message>
moving files, fixing csvs
</commit_message>
<xml_diff>
--- a/ERmodelling.xlsx
+++ b/ERmodelling.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\17900375\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tatuh\Desktop\ISYS2014 DBS\Assignment\isys2014_assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1658C8-41AE-437B-97BC-4807CA5EC72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC345365-D228-416F-9165-AE0085AEA058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{684BDCA2-E55D-4A46-B1B5-9277B055E5B1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{684BDCA2-E55D-4A46-B1B5-9277B055E5B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -415,7 +415,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,6 +619,294 @@
   </cellStyles>
   <dxfs count="74">
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -634,357 +922,67 @@
           <bgColor theme="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1052,21 +1050,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -1090,11 +1073,28 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1110,122 +1110,122 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9DA5C471-83B3-472F-827A-7DF25E73D48C}" name="Table1" displayName="Table1" ref="A11:C17" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61" headerRowBorderDxfId="73" tableBorderDxfId="72" totalsRowBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9DA5C471-83B3-472F-827A-7DF25E73D48C}" name="Table1" displayName="Table1" ref="A11:C17" totalsRowShown="0" headerRowDxfId="73" dataDxfId="71" headerRowBorderDxfId="72" tableBorderDxfId="70" totalsRowBorderDxfId="69">
   <autoFilter ref="A11:C17" xr:uid="{9DA5C471-83B3-472F-827A-7DF25E73D48C}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{5AC545D0-16D2-4088-A0E1-5606F0DC4CB6}" name="ENTITY SET" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{6B8C5329-60DE-4538-9D54-35E1FEC90B28}" name="KEY" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{AABDB00D-38D0-4013-87B8-64D4C26119B1}" name="OTHER ATTRIBUTES" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{5AC545D0-16D2-4088-A0E1-5606F0DC4CB6}" name="ENTITY SET" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{6B8C5329-60DE-4538-9D54-35E1FEC90B28}" name="KEY" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{AABDB00D-38D0-4013-87B8-64D4C26119B1}" name="OTHER ATTRIBUTES" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{B265AD4E-C631-495A-8FFB-46C6E8C10E4E}" name="Table10" displayName="Table10" ref="A21:E31" totalsRowShown="0" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{B265AD4E-C631-495A-8FFB-46C6E8C10E4E}" name="Table10" displayName="Table10" ref="A21:E31" totalsRowShown="0" dataDxfId="19">
   <autoFilter ref="A21:E31" xr:uid="{B265AD4E-C631-495A-8FFB-46C6E8C10E4E}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6B13A715-9F7D-4F7A-8239-CA048A678FD4}" name="COL NAME" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{8A721140-8714-4A9D-8997-3060701D2979}" name="TYPE" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{1DB27894-7E96-4A1F-9C0B-C22D9F130153}" name="SIZE" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{A2C92B6E-2C64-455A-A160-1F961AB1EE26}" name="NULL" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{10063662-F5FC-4648-9EEF-DFB0DC104BC0}" name="DESCRIPTION" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{6B13A715-9F7D-4F7A-8239-CA048A678FD4}" name="COL NAME" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{8A721140-8714-4A9D-8997-3060701D2979}" name="TYPE" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{1DB27894-7E96-4A1F-9C0B-C22D9F130153}" name="SIZE" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{A2C92B6E-2C64-455A-A160-1F961AB1EE26}" name="NULL" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{10063662-F5FC-4648-9EEF-DFB0DC104BC0}" name="DESCRIPTION" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{84011ED2-BDE0-4AA8-9260-39E6982D19B0}" name="Table11" displayName="Table11" ref="A41:E44" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{84011ED2-BDE0-4AA8-9260-39E6982D19B0}" name="Table11" displayName="Table11" ref="A41:E44" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A41:E44" xr:uid="{84011ED2-BDE0-4AA8-9260-39E6982D19B0}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F89F5604-39D1-4890-A3C3-4872E42948B8}" name="COL NAME" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{23EA0A37-93B0-4C79-878C-DCDBEDC15627}" name="TYPE" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4160E713-B47B-4429-B157-99D4534A0334}" name="SIZE" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{4982897B-2455-48BE-86AF-1E63383B58FE}" name="NULL" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{F40D1146-3B36-4E3E-A5D8-84B8FCF8545B}" name="DESCRIPTION" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{F89F5604-39D1-4890-A3C3-4872E42948B8}" name="COL NAME" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{23EA0A37-93B0-4C79-878C-DCDBEDC15627}" name="TYPE" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{4160E713-B47B-4429-B157-99D4534A0334}" name="SIZE" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{4982897B-2455-48BE-86AF-1E63383B58FE}" name="NULL" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{F40D1146-3B36-4E3E-A5D8-84B8FCF8545B}" name="DESCRIPTION" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{20EF3BCD-FFCB-4B4F-A030-C27AB2DD921F}" name="Table12" displayName="Table12" ref="A34:E38" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{20EF3BCD-FFCB-4B4F-A030-C27AB2DD921F}" name="Table12" displayName="Table12" ref="A34:E38" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A34:E38" xr:uid="{20EF3BCD-FFCB-4B4F-A030-C27AB2DD921F}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{93C26A6E-8F62-4F93-AD3C-BEB95DF73BAC}" name="COL NAME" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{B768F1F9-19A4-4053-ABDA-00FE4EFE5F73}" name="TYPE" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{8ADE73F1-0FCB-4666-8E2E-CBAAB15272B8}" name="SIZE" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{27428970-FBB9-44F4-B0FA-BC3740B8D3D6}" name="NULL" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{5C8A3A24-FACA-4EB8-8947-EC442C515699}" name="DESCRIPTION" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{93C26A6E-8F62-4F93-AD3C-BEB95DF73BAC}" name="COL NAME" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{B768F1F9-19A4-4053-ABDA-00FE4EFE5F73}" name="TYPE" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{8ADE73F1-0FCB-4666-8E2E-CBAAB15272B8}" name="SIZE" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{27428970-FBB9-44F4-B0FA-BC3740B8D3D6}" name="NULL" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{5C8A3A24-FACA-4EB8-8947-EC442C515699}" name="DESCRIPTION" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{9ED3A770-9A9B-4AF4-86B1-A34A9CF5B0C7}" name="Table6" displayName="Table6" ref="A3:C9" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{9ED3A770-9A9B-4AF4-86B1-A34A9CF5B0C7}" name="Table6" displayName="Table6" ref="A3:C9" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A3:C9" xr:uid="{9ED3A770-9A9B-4AF4-86B1-A34A9CF5B0C7}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{C4E994CF-6698-43FC-8034-5AE0A62F757B}" name="ENTITY SET" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{8778C0D8-58CA-45B5-BDAA-EA67AFDEE8AD}" name="KEY" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{7EDAB2D7-2527-4E78-9042-88C10168C22A}" name="OTHER ATTRIBUTES" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{C4E994CF-6698-43FC-8034-5AE0A62F757B}" name="ENTITY SET" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{8778C0D8-58CA-45B5-BDAA-EA67AFDEE8AD}" name="KEY" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{7EDAB2D7-2527-4E78-9042-88C10168C22A}" name="OTHER ATTRIBUTES" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1D7DADBC-0C72-446F-97CA-BB1D311CBDDE}" name="Table2" displayName="Table2" ref="A47:E50" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1D7DADBC-0C72-446F-97CA-BB1D311CBDDE}" name="Table2" displayName="Table2" ref="A47:E50" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59">
   <autoFilter ref="A47:E50" xr:uid="{1D7DADBC-0C72-446F-97CA-BB1D311CBDDE}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D34C4BBA-FD13-4F30-B8F2-72898F3B61A4}" name="COLNAME" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{22F88310-673C-4C9F-99AC-00AD66346E40}" name="TYPE" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{1F306150-308E-465F-9CBF-936875CC5F25}" name="SIZE" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{32FC0437-BDC7-45A5-ADA9-CF13B314F6C4}" name="NULL" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{F720693E-E73B-4D47-9C3B-B2417D5F690A}" name="DESCRIPTION" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D34C4BBA-FD13-4F30-B8F2-72898F3B61A4}" name="COLNAME" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{22F88310-673C-4C9F-99AC-00AD66346E40}" name="TYPE" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{1F306150-308E-465F-9CBF-936875CC5F25}" name="SIZE" dataDxfId="56"/>
+    <tableColumn id="4" xr3:uid="{32FC0437-BDC7-45A5-ADA9-CF13B314F6C4}" name="NULL" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{F720693E-E73B-4D47-9C3B-B2417D5F690A}" name="DESCRIPTION" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C0EAEE3C-2D0E-4343-A6DC-A92A3E98271F}" name="Table3" displayName="Table3" ref="A53:E62" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C0EAEE3C-2D0E-4343-A6DC-A92A3E98271F}" name="Table3" displayName="Table3" ref="A53:E62" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A53:E62" xr:uid="{C0EAEE3C-2D0E-4343-A6DC-A92A3E98271F}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{14577A3A-F5CE-4078-B482-C688F693F948}" name="COLNAME" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{53320488-D7A7-484A-851D-5042F589884D}" name="TYPE" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{887E2941-DB2B-4C69-942F-C03CB1304CF5}" name="SIZE" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{7AA6EC6E-FC7E-4984-803B-DBC0D1EB1B02}" name="NULL" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{B025FFA2-46DF-4614-AA9A-BF2722B5DFBD}" name="DESCRIPTION" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{14577A3A-F5CE-4078-B482-C688F693F948}" name="COLNAME" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{53320488-D7A7-484A-851D-5042F589884D}" name="TYPE" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{887E2941-DB2B-4C69-942F-C03CB1304CF5}" name="SIZE" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{7AA6EC6E-FC7E-4984-803B-DBC0D1EB1B02}" name="NULL" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{B025FFA2-46DF-4614-AA9A-BF2722B5DFBD}" name="DESCRIPTION" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5F142F14-6FD0-4F75-96CC-DD57F4634499}" name="Table4" displayName="Table4" ref="A65:E72" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5F142F14-6FD0-4F75-96CC-DD57F4634499}" name="Table4" displayName="Table4" ref="A65:E72" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A65:E72" xr:uid="{5F142F14-6FD0-4F75-96CC-DD57F4634499}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{89764756-3D13-4D4E-B592-CD960020956A}" name="COLNAME" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{C08162E3-666D-4AE3-9823-05297074E9DB}" name="TYPE" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{E60D850D-5D0E-4AA9-BA9B-530054EFDAAB}" name="SIZE" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{047B97D9-4127-4EC9-8006-913CA660CC98}" name="NULL" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{B517EB3D-D996-49A5-950E-97AF72BE25E8}" name="DESCRIPTION" dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{89764756-3D13-4D4E-B592-CD960020956A}" name="COLNAME" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{C08162E3-666D-4AE3-9823-05297074E9DB}" name="TYPE" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{E60D850D-5D0E-4AA9-BA9B-530054EFDAAB}" name="SIZE" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{047B97D9-4127-4EC9-8006-913CA660CC98}" name="NULL" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{B517EB3D-D996-49A5-950E-97AF72BE25E8}" name="DESCRIPTION" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5AAA0A74-0852-421F-9BCD-356F1D9E7E22}" name="Table5" displayName="Table5" ref="A75:E78" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5AAA0A74-0852-421F-9BCD-356F1D9E7E22}" name="Table5" displayName="Table5" ref="A75:E78" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A75:E78" xr:uid="{5AAA0A74-0852-421F-9BCD-356F1D9E7E22}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{89368BF0-F206-40E1-A587-D3AD345772D9}" name="COLNAME" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{C51DA079-A48C-4C6E-84AE-150F25EEB8BE}" name="TYPE" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{3B689567-58A9-4324-BD9A-71F82ED79D51}" name="SIZE" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{1BB841EE-BB1C-4F20-98AA-E8CAE0727EEE}" name="NULL" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{FD1ED0CC-B42E-45C9-8CAE-DE4DF367EBE6}" name="DESCRIPTION" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{89368BF0-F206-40E1-A587-D3AD345772D9}" name="COLNAME" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{C51DA079-A48C-4C6E-84AE-150F25EEB8BE}" name="TYPE" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{3B689567-58A9-4324-BD9A-71F82ED79D51}" name="SIZE" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{1BB841EE-BB1C-4F20-98AA-E8CAE0727EEE}" name="NULL" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{FD1ED0CC-B42E-45C9-8CAE-DE4DF367EBE6}" name="DESCRIPTION" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1246,28 +1246,28 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CD277794-A816-48EA-B99F-E172EB200DF7}" name="Table8" displayName="Table8" ref="A10:E13" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CD277794-A816-48EA-B99F-E172EB200DF7}" name="Table8" displayName="Table8" ref="A10:E13" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A10:E13" xr:uid="{CD277794-A816-48EA-B99F-E172EB200DF7}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{92D36599-B36C-4454-9560-EF797281B66A}" name="COL NAME" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{990036EB-804C-4A5B-BE86-B5E380C767D2}" name="TYPE" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{D521F45C-A31D-4D0C-8585-AF41AD783090}" name="SIZE" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{DEA966A5-AF7E-46C9-A3BD-D63F8137B3D9}" name="NULL" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{14F55298-EA3E-4674-BCA1-2FF812B36D13}" name="DESCRIPTION" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{92D36599-B36C-4454-9560-EF797281B66A}" name="COL NAME" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{990036EB-804C-4A5B-BE86-B5E380C767D2}" name="TYPE" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{D521F45C-A31D-4D0C-8585-AF41AD783090}" name="SIZE" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{DEA966A5-AF7E-46C9-A3BD-D63F8137B3D9}" name="NULL" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{14F55298-EA3E-4674-BCA1-2FF812B36D13}" name="DESCRIPTION" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{5165DA44-BB3D-4EC5-986B-510B0F417013}" name="Table9" displayName="Table9" ref="A16:E18" totalsRowShown="0" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{5165DA44-BB3D-4EC5-986B-510B0F417013}" name="Table9" displayName="Table9" ref="A16:E18" totalsRowShown="0" dataDxfId="25">
   <autoFilter ref="A16:E18" xr:uid="{5165DA44-BB3D-4EC5-986B-510B0F417013}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{15EA0CD8-A860-4C3D-8AD6-D9E20612D4CD}" name="COL NAME" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{39DCCE42-6B06-4856-AA18-77B3C3176B77}" name="TYPE" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{B63DD618-A79D-4307-8FF4-1FE534D0DB87}" name="SIZE" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{49B0A964-1D8D-4AC3-A8A4-5E3CE5EA22B8}" name="NULL" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{EC0965AE-360D-4BF0-8A19-F84631A26B2A}" name="DESCRIPTION" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{15EA0CD8-A860-4C3D-8AD6-D9E20612D4CD}" name="COL NAME" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{39DCCE42-6B06-4856-AA18-77B3C3176B77}" name="TYPE" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{B63DD618-A79D-4307-8FF4-1FE534D0DB87}" name="SIZE" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{49B0A964-1D8D-4AC3-A8A4-5E3CE5EA22B8}" name="NULL" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{EC0965AE-360D-4BF0-8A19-F84631A26B2A}" name="DESCRIPTION" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1591,24 +1591,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B48B21F7-D6DE-4CAE-B44F-1848A06C4887}">
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.125" customWidth="1"/>
-    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.375" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>76</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="42.75">
+    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>68</v>
       </c>
@@ -1663,7 +1663,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="28.5">
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>81</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" s="1" customFormat="1">
+    <row r="12" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>3</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:3" s="1" customFormat="1">
+    <row r="13" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>36</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:3" s="1" customFormat="1" ht="42.75">
+    <row r="14" spans="1:3" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>68</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:3" s="1" customFormat="1">
+    <row r="15" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>6</v>
       </c>
@@ -1740,12 +1740,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" s="1" customFormat="1">
+    <row r="16" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
     </row>
-    <row r="17" spans="1:3" s="1" customFormat="1" ht="28.5">
+    <row r="17" spans="1:3" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>53</v>
       </c>
@@ -1756,32 +1756,32 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1799,23 +1799,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A33870-F9C9-4E60-ACDD-862C7BBB12D9}">
   <dimension ref="A1:E78"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.125" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>83</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1880,12 +1880,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>83</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>69</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>88</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="28.5">
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>90</v>
       </c>
@@ -1953,12 +1953,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>83</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>77</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="28.5">
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>78</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>27</v>
       </c>
       <c r="C18" s="3">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>28</v>
@@ -2009,12 +2009,12 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>83</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="28.5">
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="28.5">
+    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>97</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="28.5">
+    <row r="24" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>85</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="28.5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>101</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="28.5">
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>103</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>39</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="28.5">
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>105</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>108</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>111</v>
       </c>
@@ -2187,12 +2187,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>83</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>72</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>114</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>116</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="28.5">
+    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>103</v>
       </c>
@@ -2273,12 +2273,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>83</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>10</v>
       </c>
@@ -2312,7 +2312,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>5</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="28.5">
+    <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>42</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>3</v>
       </c>
@@ -2355,7 +2355,7 @@
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
     </row>
-    <row r="47" spans="1:5" ht="15">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
         <v>19</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>10</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>26</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>30</v>
       </c>
@@ -2421,14 +2421,14 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="14"/>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
     </row>
-    <row r="52" spans="1:5" ht="15">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
         <v>4</v>
       </c>
@@ -2437,7 +2437,7 @@
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
     </row>
-    <row r="53" spans="1:5" ht="15">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>19</v>
       </c>
@@ -2454,7 +2454,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
         <v>5</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="28.5">
+    <row r="55" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
         <v>33</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="28.5">
+    <row r="56" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
         <v>34</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="28.5">
+    <row r="57" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>36</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="28.5">
+    <row r="58" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
         <v>39</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="28.5">
+    <row r="59" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>42</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="28.5">
+    <row r="60" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>45</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
         <v>48</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
         <v>51</v>
       </c>
@@ -2595,14 +2595,14 @@
         <v>52</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="14"/>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
       <c r="E63" s="14"/>
     </row>
-    <row r="64" spans="1:5" ht="15">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
         <v>53</v>
       </c>
@@ -2611,7 +2611,7 @@
       <c r="D64" s="14"/>
       <c r="E64" s="14"/>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
         <v>19</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="16" t="s">
         <v>9</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="28.5">
+    <row r="67" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="16" t="s">
         <v>36</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="28.5">
+    <row r="68" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="16" t="s">
         <v>56</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="28.5">
+    <row r="69" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="16" t="s">
         <v>57</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="28.5">
+    <row r="70" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="16" t="s">
         <v>58</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="28.5">
+    <row r="71" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="16" t="s">
         <v>59</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="28.5">
+    <row r="72" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="16" t="s">
         <v>60</v>
       </c>
@@ -2737,14 +2737,14 @@
         <v>61</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="14"/>
       <c r="B73" s="14"/>
       <c r="C73" s="14"/>
       <c r="D73" s="14"/>
       <c r="E73" s="14"/>
     </row>
-    <row r="74" spans="1:5" ht="15">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
         <v>6</v>
       </c>
@@ -2753,7 +2753,7 @@
       <c r="D74" s="14"/>
       <c r="E74" s="14"/>
     </row>
-    <row r="75" spans="1:5" ht="15">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="16" t="s">
         <v>19</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="16" t="s">
         <v>10</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="16" t="s">
         <v>5</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="28.5">
+    <row r="78" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="16" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
chaning avg rating to decimal(3,1)
</commit_message>
<xml_diff>
--- a/ERmodelling.xlsx
+++ b/ERmodelling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tatuh\Desktop\ISYS2014 DBS\Assignment\isys2014_assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC345365-D228-416F-9165-AE0085AEA058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA5E97B-7B73-49A6-ABDC-C4443B391F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{684BDCA2-E55D-4A46-B1B5-9277B055E5B1}"/>
   </bookViews>
@@ -396,9 +396,6 @@
     <t>sum of ticket price</t>
   </si>
   <si>
-    <t>(1,2)</t>
-  </si>
-  <si>
     <t>average of rating of the tour package</t>
   </si>
   <si>
@@ -409,6 +406,9 @@
   </si>
   <si>
     <t>rating of the tourit attraction</t>
+  </si>
+  <si>
+    <t>(3,1)</t>
   </si>
 </sst>
 </file>
@@ -2120,7 +2120,7 @@
         <v>40</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
@@ -2266,16 +2266,16 @@
         <v>40</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2326,7 +2326,7 @@
         <v>28</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -2343,7 +2343,7 @@
         <v>28</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
minimum of part4 is done
</commit_message>
<xml_diff>
--- a/ERmodelling.xlsx
+++ b/ERmodelling.xlsx
@@ -781,7 +781,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.28"/>
@@ -997,7 +997,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E1048576"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.15"/>
@@ -1254,7 +1254,7 @@
         <v>50</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>41</v>

</xml_diff>